<commit_message>
file pptx và test case hoàn chỉnh
</commit_message>
<xml_diff>
--- a/Extra/testcase.xlsx
+++ b/Extra/testcase.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\hoctap\Lập Trình Mạng\Ung-Dung-ChatTCP\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F153401C-0A61-4EC2-BD69-3520C266BAC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9BCC649-92E3-4A89-972E-2A45F482B6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="125">
   <si>
     <t>STT(Mã TC)</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>Kết quả mong đợi(Expected result)</t>
-  </si>
-  <si>
-    <t>Trạng thái(Status)</t>
   </si>
   <si>
     <t>TC_01</t>
@@ -422,6 +419,25 @@
 Kết quả ImageTC-18+1
 ImageTC-18+2
 Kết quả ImageTC-18+2</t>
+  </si>
+  <si>
+    <t>Trạng thái 1(Status)</t>
+  </si>
+  <si>
+    <t>Trạng thái 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client chạy song song với Server thì Port chỉ nhận số 5000, nếu nhập số khác 5000 và nhập chữ thì sẽ hiện thông báo:"không thể kết nối tới Server </t>
+  </si>
+  <si>
+    <t>Sau khi nhận tin nhắn mà chưa đọc thì khi tải lại lịch sử sẽ hiện lên tổng tin nhắn đã nhận bao gồm tin nhắn cũ và mới</t>
+  </si>
+  <si>
+    <t>Sau khi nhấn đăng xuất thì sẽ quay lại Client đăng nhập để truy cập vào tài khoản</t>
+  </si>
+  <si>
+    <t>ImageTC-16
+Kết quả ImageTC-16</t>
   </si>
 </sst>
 </file>
@@ -476,7 +492,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -536,18 +552,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -557,33 +636,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -592,13 +644,436 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="13">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -609,6 +1084,26 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4EF12B6-01F3-4FF6-8086-2D3505551CD1}" name="Table1" displayName="Table1" ref="A1:K20" totalsRowShown="0" headerRowBorderDxfId="11" tableBorderDxfId="12">
+  <autoFilter ref="A1:K20" xr:uid="{C4EF12B6-01F3-4FF6-8086-2D3505551CD1}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{407C634F-38BB-4D5D-9759-A22BBD583538}" name="STT(Mã TC)" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{1EBF301C-9DE5-452C-89AE-63AB3CE65E32}" name="Chức năng cần test" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{03379C37-9C01-431D-A3E0-A8B971C4BB14}" name="Các bước thực hiện(Steps)" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{2DB51D45-B1C7-42CE-9119-C1E5AB63EDE8}" name="Dữ liệu nhập vào(Test Data)" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{E50E6BD6-D1D4-43C1-ADB7-3CE2ED80FE38}" name="Kết quả mong đợi(Expected result)" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{EE302A62-431E-4E85-8EE6-BC4A1F60B45D}" name="Test1" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{AF489F94-995E-4928-BF96-0D915FCB5BB9}" name="Test2" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{171F06EA-4E90-4D7A-87FB-B1EFBDE98621}" name="Test 3" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{6D6445E0-5FA8-492F-B9CD-123B33DF2171}" name="Trạng thái 1(Status)" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{95887B5A-2564-4A33-BE00-9933053326C5}" name="Trạng thái 2" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{20C69844-8620-4CC8-919A-69588876071C}" name="Proof" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -931,575 +1426,606 @@
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.109375" style="2"/>
+    <col min="1" max="1" width="13.88671875" style="2" customWidth="1"/>
     <col min="2" max="2" width="26" style="2" customWidth="1"/>
-    <col min="3" max="3" width="25.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.77734375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="27.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33" style="2" customWidth="1"/>
     <col min="6" max="6" width="21.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.5546875" style="26" customWidth="1"/>
     <col min="8" max="8" width="8.88671875" style="2"/>
-    <col min="9" max="9" width="8.88671875" style="1"/>
-    <col min="10" max="10" width="21.109375" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="1"/>
+    <col min="9" max="9" width="20.109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.77734375" customWidth="1"/>
+    <col min="11" max="11" width="21.109375" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H1" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="I1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J1" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="K1" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="69" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="K1" s="4"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="6"/>
+      <c r="K2" s="11" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" ht="110.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="5" t="s">
+    <row r="3" spans="1:11" ht="138" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="K2" s="4"/>
+      <c r="K3" s="12" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" ht="220.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="5" t="s">
+    <row r="4" spans="1:11" ht="96.6" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="J3" s="15" t="s">
+      <c r="B4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="4"/>
+      <c r="F4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="8"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J4" s="6"/>
+      <c r="K4" s="13" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" ht="124.2" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5" t="s">
+    <row r="5" spans="1:11" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="7" t="s">
+      <c r="B5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="8"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="10"/>
+    </row>
+    <row r="6" spans="1:11" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="4"/>
+      <c r="I6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="6"/>
+      <c r="K6" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="K4" s="4"/>
     </row>
-    <row r="5" spans="1:11" ht="69" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="5" t="s">
+    <row r="7" spans="1:11" ht="41.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="13"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" s="6"/>
+      <c r="K7" s="13" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" ht="82.8" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="K6" s="4"/>
+    <row r="8" spans="1:11" ht="55.2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="13" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="7" spans="1:11" ht="69" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="13"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="K7" s="4"/>
-    </row>
-    <row r="8" spans="1:11" ht="69" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="9" spans="1:11" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="K8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" ht="55.2" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="B9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="C9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="10"/>
     </row>
     <row r="10" spans="1:11" ht="70.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J10" s="16" t="s">
+      <c r="F10" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="124.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" spans="1:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="B11" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="4"/>
+      <c r="E11" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="G11" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="H11" s="4"/>
+      <c r="I11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11" s="10"/>
     </row>
     <row r="12" spans="1:11" ht="118.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="F12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:11" ht="67.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="D13" s="7"/>
+      <c r="E13" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17" t="s">
+      <c r="F13" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="G13" s="8"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="G13" s="18"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J13" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="K13" s="16"/>
     </row>
     <row r="14" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="C14" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="D14" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="E14" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="F14" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="G14" s="8"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="6"/>
+      <c r="K14" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="G14" s="18"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J14" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="K14" s="16"/>
     </row>
     <row r="15" spans="1:11" ht="65.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="C15" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="D15" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="E15" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="F15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G15" s="18"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J15" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="K15" s="16"/>
     </row>
     <row r="16" spans="1:11" ht="76.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="D16" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="E16" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E16" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="18"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="F16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J16" s="6"/>
+      <c r="K16" s="14"/>
     </row>
-    <row r="17" spans="1:11" ht="55.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+    <row r="17" spans="1:11" ht="85.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="C17" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="D17" s="7"/>
+      <c r="E17" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17" t="s">
+      <c r="F17" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F17" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="G17" s="18"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="16" t="s">
-        <v>47</v>
-      </c>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
+      <c r="G17" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="C18" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="D18" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="E18" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="F18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="8"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" s="6"/>
+      <c r="K18" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="F18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G18" s="18"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J18" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="K18" s="16"/>
     </row>
     <row r="19" spans="1:11" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="C19" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="D19" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="E19" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="F19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G19" s="8"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J19" s="6"/>
+      <c r="K19" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="F19" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G19" s="18"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="J19" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="K19" s="16"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="20"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="22"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1:K20">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="J4" r:id="rId1" xr:uid="{5948687F-5235-4C94-B690-0DC336279BA8}"/>
-    <hyperlink ref="J6" r:id="rId2" xr:uid="{357784ED-03BA-48CB-A0E8-094DA2F96A04}"/>
-    <hyperlink ref="J7" r:id="rId3" xr:uid="{9B2DD5E7-BECF-424E-A92A-7BD32D6ABFCD}"/>
-    <hyperlink ref="J8" r:id="rId4" xr:uid="{A67FC0FE-3B01-4960-820B-6B72C7CE3EE1}"/>
-    <hyperlink ref="J12" r:id="rId5" xr:uid="{F2730E77-2212-4681-9F73-C4C0A739E663}"/>
-    <hyperlink ref="J14" r:id="rId6" xr:uid="{DAE379E1-CC8D-4407-B295-2006C3968641}"/>
-    <hyperlink ref="J15" r:id="rId7" xr:uid="{BD6E9BFA-15C4-4CDB-B8B1-4DCF4A455B17}"/>
+    <hyperlink ref="K15" r:id="rId1" xr:uid="{BD6E9BFA-15C4-4CDB-B8B1-4DCF4A455B17}"/>
+    <hyperlink ref="K14" r:id="rId2" xr:uid="{DAE379E1-CC8D-4407-B295-2006C3968641}"/>
+    <hyperlink ref="K12" r:id="rId3" xr:uid="{F2730E77-2212-4681-9F73-C4C0A739E663}"/>
+    <hyperlink ref="K8" r:id="rId4" xr:uid="{A67FC0FE-3B01-4960-820B-6B72C7CE3EE1}"/>
+    <hyperlink ref="K7" r:id="rId5" xr:uid="{9B2DD5E7-BECF-424E-A92A-7BD32D6ABFCD}"/>
+    <hyperlink ref="K6" r:id="rId6" xr:uid="{357784ED-03BA-48CB-A0E8-094DA2F96A04}"/>
+    <hyperlink ref="K4" r:id="rId7" xr:uid="{5948687F-5235-4C94-B690-0DC336279BA8}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId8"/>
+  <tableParts count="1">
+    <tablePart r:id="rId9"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>